<commit_message>
#5 Client and eSpark BOM Update peripherals remaining.
</commit_message>
<xml_diff>
--- a/Design files/Left-Side/BOM/Client BOM-LEFT-Bone_Conduction_Glasses.xlsx
+++ b/Design files/Left-Side/BOM/Client BOM-LEFT-Bone_Conduction_Glasses.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="141">
   <si>
     <t>#</t>
   </si>
@@ -39,15 +39,9 @@
     <t>Ferrite Bead</t>
   </si>
   <si>
-    <t>Test Point</t>
-  </si>
-  <si>
     <t>USB B Connector</t>
   </si>
   <si>
-    <t>SMD Pads</t>
-  </si>
-  <si>
     <t>Inductor</t>
   </si>
   <si>
@@ -60,9 +54,6 @@
     <t>Variable Resistor</t>
   </si>
   <si>
-    <t>Solder Bridge</t>
-  </si>
-  <si>
     <t>Switch</t>
   </si>
   <si>
@@ -102,18 +93,9 @@
     <t>FB1, FB2</t>
   </si>
   <si>
-    <t>J1, J4</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
-    <t>J3</t>
-  </si>
-  <si>
-    <t>J5</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -126,9 +108,6 @@
     <t>LED2</t>
   </si>
   <si>
-    <t>P1, P2, P3</t>
-  </si>
-  <si>
     <t>R1, R6</t>
   </si>
   <si>
@@ -144,9 +123,6 @@
     <t>R12</t>
   </si>
   <si>
-    <t>SB1, SB2, SB3, SB4, SB5, SB6, SB7, SB8, SB9, SB10, SB11, SB12, SB13, SB14</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -192,15 +168,9 @@
     <t>FERRITE BEAD 220 OHM 0603 1LN</t>
   </si>
   <si>
-    <t>Wire Connecting Pad</t>
-  </si>
-  <si>
     <t>CONN RCPT USB2.0 MICRO B SMD R/A</t>
   </si>
   <si>
-    <t>Wire Connecting Pads</t>
-  </si>
-  <si>
     <t>FIXED IND 2.7NH 500MA 200MOHM SM</t>
   </si>
   <si>
@@ -213,9 +183,6 @@
     <t>RED LED 0603 Light Emitting Diodes</t>
   </si>
   <si>
-    <t>Test Point ON</t>
-  </si>
-  <si>
     <t>RES 1K OHM 1% 1/20W 0201</t>
   </si>
   <si>
@@ -231,9 +198,6 @@
     <t>TRIMMER 1M OHM 0.1W J LEAD TOP</t>
   </si>
   <si>
-    <t>Solder Bridge ON</t>
-  </si>
-  <si>
     <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
   </si>
   <si>
@@ -270,30 +234,18 @@
     <t>IND-0603 (1608 Metric)</t>
   </si>
   <si>
-    <t>2 Test Pad</t>
-  </si>
-  <si>
-    <t>5 Test Pad</t>
-  </si>
-  <si>
     <t>IND-0201</t>
   </si>
   <si>
     <t>LED-0603</t>
   </si>
   <si>
-    <t>Test-point - 0.5mm</t>
-  </si>
-  <si>
     <t>Res-0201</t>
   </si>
   <si>
     <t>TC33X-2-105E</t>
   </si>
   <si>
-    <t>Solder Bridge 0402</t>
-  </si>
-  <si>
     <t>B3U-1000P</t>
   </si>
   <si>
@@ -337,9 +289,6 @@
   </si>
   <si>
     <t>10118194-0001LF</t>
-  </si>
-  <si>
-    <t>4 Pin SMD Wire Connector</t>
   </si>
   <si>
     <t>LQP03TN2N7B02D</t>
@@ -680,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -717,9 +666,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -729,6 +675,26 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1016,7 +982,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1041,10 +1007,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1055,31 +1021,31 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>149</v>
+        <v>132</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>151</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1092,22 +1058,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="J3" s="7">
         <v>1</v>
@@ -1121,35 +1087,35 @@
     <row r="4" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B32" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B27" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="J4" s="9">
         <v>18</v>
       </c>
       <c r="K4" s="7">
-        <f t="shared" ref="K4:K33" si="1">J4*5</f>
+        <f t="shared" ref="K4:K26" si="1">J4*5</f>
         <v>90</v>
       </c>
       <c r="L4" s="9"/>
@@ -1164,22 +1130,22 @@
         <v>3</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
       <c r="J5" s="7">
         <v>6</v>
@@ -1200,22 +1166,22 @@
         <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
@@ -1236,22 +1202,22 @@
         <v>3</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1272,22 +1238,22 @@
         <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1308,22 +1274,22 @@
         <v>3</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -1344,22 +1310,22 @@
         <v>4</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="J10" s="9">
         <v>4</v>
@@ -1380,22 +1346,22 @@
         <v>5</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="J11" s="7">
         <v>2</v>
@@ -1409,180 +1375,182 @@
     <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
+        <f>ROW(B12) - ROW($B$2)</f>
+        <v>10</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="J12" s="7">
+        <v>1</v>
+      </c>
+      <c r="K12" s="7">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L12" s="7"/>
+    </row>
+    <row r="13" spans="1:12" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="18"/>
+      <c r="B13" s="19">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J12" s="9">
-        <v>2</v>
-      </c>
-      <c r="K12" s="7">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="L12" s="9"/>
-    </row>
-    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="11">
-        <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="I13" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J13" s="7">
+      <c r="D13" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="I13" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="J13" s="21">
         <v>1</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="23">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L13" s="7"/>
+      <c r="L13" s="21"/>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B14) - ROW($B$2)</f>
         <v>12</v>
       </c>
-      <c r="C14" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>57</v>
+      <c r="C14" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J14" s="9">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="7">
+        <v>2</v>
       </c>
       <c r="K14" s="7">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="L14" s="9"/>
-    </row>
-    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="L14" s="7"/>
+    </row>
+    <row r="15" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="11">
-        <f>ROW(B15) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>154</v>
+      <c r="D15" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>110</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J15" s="7">
+        <v>124</v>
+      </c>
+      <c r="J15" s="9">
         <v>1</v>
       </c>
       <c r="K15" s="7">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L15" s="7"/>
+      <c r="L15" s="9"/>
     </row>
     <row r="16" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B16) - ROW($B$2)</f>
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="J16" s="9">
+      <c r="C16" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="J16" s="7">
         <v>1</v>
       </c>
       <c r="K16" s="7">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L16" s="9"/>
+      <c r="L16" s="7"/>
     </row>
     <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -1590,26 +1558,26 @@
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="13" t="s">
         <v>9</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -1620,75 +1588,75 @@
       </c>
       <c r="L17" s="7"/>
     </row>
-    <row r="18" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="J18" s="9">
+        <v>2</v>
+      </c>
+      <c r="K18" s="7">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="I18" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="J18" s="9">
-        <v>1</v>
-      </c>
-      <c r="K18" s="7">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
       <c r="L18" s="9"/>
     </row>
-    <row r="19" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="J19" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K19" s="7">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L19" s="7"/>
     </row>
@@ -1699,32 +1667,32 @@
         <v>18</v>
       </c>
       <c r="C20" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="I20" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="J20" s="9">
         <v>6</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J20" s="9">
-        <v>3</v>
-      </c>
       <c r="K20" s="7">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="L20" s="9"/>
     </row>
@@ -1734,181 +1702,181 @@
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="13" t="s">
-        <v>11</v>
+      <c r="C21" s="12" t="s">
+        <v>10</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="G21" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="H21" s="7" t="s">
-        <v>121</v>
-      </c>
       <c r="I21" s="8" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="J21" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L21" s="7"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B22) - ROW($B$2)</f>
         <v>20</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="G22" s="10" t="s">
+      <c r="D22" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="H22" s="9" t="s">
-        <v>121</v>
-      </c>
       <c r="I22" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="J22" s="9">
-        <v>2</v>
+        <v>137</v>
+      </c>
+      <c r="J22" s="7">
+        <v>1</v>
       </c>
       <c r="K22" s="7">
         <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="L22" s="9"/>
+        <v>5</v>
+      </c>
+      <c r="L22" s="7"/>
     </row>
     <row r="23" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
-        <f>ROW(B23) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C23" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G23" s="8" t="s">
+      <c r="C23" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="H23" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="J23" s="7">
-        <v>3</v>
+      <c r="I23" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="J23" s="9">
+        <v>1</v>
       </c>
       <c r="K23" s="7">
         <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="L23" s="7"/>
+        <v>5</v>
+      </c>
+      <c r="L23" s="9"/>
     </row>
     <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B24) - ROW($B$2)</f>
         <v>22</v>
       </c>
-      <c r="C24" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="G24" s="10" t="s">
+      <c r="C24" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H24" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="H24" s="9" t="s">
-        <v>121</v>
-      </c>
       <c r="I24" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="J24" s="9">
-        <v>6</v>
+        <v>137</v>
+      </c>
+      <c r="J24" s="7">
+        <v>1</v>
       </c>
       <c r="K24" s="7">
         <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="L24" s="9"/>
+        <v>5</v>
+      </c>
+      <c r="L24" s="7"/>
     </row>
     <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
-        <f>ROW(B25) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="J25" s="7">
+      <c r="D25" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="J25" s="9">
         <v>1</v>
       </c>
       <c r="K25" s="7">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L25" s="7"/>
-    </row>
-    <row r="26" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L25" s="9"/>
+    </row>
+    <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
@@ -1918,261 +1886,81 @@
         <v>13</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>153</v>
+        <v>63</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>154</v>
+        <v>106</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="J26" s="9">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="K26" s="7">
         <f t="shared" si="1"/>
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="L26" s="9"/>
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
-        <f>ROW(B27) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C27" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>153</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>129</v>
-      </c>
+      <c r="C27" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="10"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="H27" s="9"/>
       <c r="I27" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J27" s="7">
-        <v>1</v>
-      </c>
-      <c r="K27" s="7">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="L27" s="7"/>
+        <v>137</v>
+      </c>
+      <c r="J27" s="9"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="9"/>
     </row>
     <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B28) - ROW($B$2)</f>
         <v>26</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>115</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>130</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J28" s="9">
-        <v>1</v>
-      </c>
-      <c r="K28" s="7">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="L28" s="9"/>
-    </row>
-    <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
-      <c r="B29" s="11">
-        <f>ROW(B29) - ROW($B$2)</f>
-        <v>27</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="I29" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J29" s="7">
-        <v>1</v>
-      </c>
-      <c r="K29" s="7">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="L29" s="7"/>
-    </row>
-    <row r="30" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="1"/>
-      <c r="B30" s="11">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J30" s="9">
-        <v>1</v>
-      </c>
-      <c r="K30" s="7">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="L30" s="9"/>
-    </row>
-    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="1"/>
-      <c r="B31" s="11">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="G31" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="I31" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="J31" s="9">
-        <v>1</v>
-      </c>
-      <c r="K31" s="7">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="L31" s="9"/>
-    </row>
-    <row r="32" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="1"/>
-      <c r="B32" s="11">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="E32" s="10"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="H32" s="9"/>
-      <c r="I32" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="J32" s="9"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="9"/>
-    </row>
-    <row r="33" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="1"/>
-      <c r="B33" s="11">
-        <f>ROW(B33) - ROW($B$2)</f>
-        <v>31</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="E33" s="17"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="H33" s="16"/>
-      <c r="I33" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
+      <c r="C28" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" s="16"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="H28" s="15"/>
+      <c r="I28" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="J28" s="15"/>
+      <c r="K28" s="15"/>
+      <c r="L28" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
#5 eSpark and Client BOM Updated with mention Peripheral in Skype group
</commit_message>
<xml_diff>
--- a/Design files/Left-Side/BOM/Client BOM-LEFT-Bone_Conduction_Glasses.xlsx
+++ b/Design files/Left-Side/BOM/Client BOM-LEFT-Bone_Conduction_Glasses.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="143">
   <si>
     <t>#</t>
   </si>
@@ -441,7 +441,13 @@
     <t>Battery</t>
   </si>
   <si>
-    <t>Transducer</t>
+    <t>3.7V Lithium Polymer Rechargeable Battery 501230 300mah</t>
+  </si>
+  <si>
+    <t>Bone Conduction Module Sensor Deafness Dumb Mini bone conduction horn speaker (GD02)</t>
+  </si>
+  <si>
+    <t>Transducer (GD02)</t>
   </si>
 </sst>
 </file>
@@ -675,9 +681,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -695,6 +698,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1007,10 +1013,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1115,7 +1121,7 @@
         <v>18</v>
       </c>
       <c r="K4" s="7">
-        <f t="shared" ref="K4:K26" si="1">J4*5</f>
+        <f t="shared" ref="K4:K28" si="1">J4*5</f>
         <v>90</v>
       </c>
       <c r="L4" s="9"/>
@@ -1408,41 +1414,41 @@
       </c>
       <c r="L12" s="7"/>
     </row>
-    <row r="13" spans="1:12" s="24" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="18"/>
-      <c r="B13" s="19">
+    <row r="13" spans="1:12" s="23" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="17"/>
+      <c r="B13" s="18">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="21" t="s">
+      <c r="D13" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="22" t="s">
+      <c r="E13" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="F13" s="21" t="s">
+      <c r="F13" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="I13" s="22" t="s">
+      <c r="I13" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="20">
         <v>1</v>
       </c>
-      <c r="K13" s="23">
+      <c r="K13" s="22">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="L13" s="21"/>
+      <c r="L13" s="20"/>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -1912,7 +1918,7 @@
       </c>
       <c r="L26" s="9"/>
     </row>
-    <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
         <f t="shared" si="0"/>
@@ -1924,20 +1930,30 @@
       <c r="D27" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E27" s="10"/>
-      <c r="F27" s="9"/>
+      <c r="E27" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>137</v>
+      </c>
       <c r="G27" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="H27" s="9"/>
+      <c r="H27" s="9" t="s">
+        <v>137</v>
+      </c>
       <c r="I27" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="J27" s="9"/>
-      <c r="K27" s="7"/>
+      <c r="J27" s="9">
+        <v>1</v>
+      </c>
+      <c r="K27" s="7">
+        <v>5</v>
+      </c>
       <c r="L27" s="9"/>
     </row>
-    <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f>ROW(B28) - ROW($B$2)</f>
@@ -1949,17 +1965,27 @@
       <c r="D28" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="E28" s="16"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="H28" s="15"/>
+      <c r="E28" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="H28" s="15" t="s">
+        <v>137</v>
+      </c>
       <c r="I28" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
+      <c r="J28" s="15">
+        <v>1</v>
+      </c>
+      <c r="K28" s="15">
+        <v>5</v>
+      </c>
       <c r="L28" s="15"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#5 Touch material peripheral added in BOMs.
</commit_message>
<xml_diff>
--- a/Design files/Left-Side/BOM/Client BOM-LEFT-Bone_Conduction_Glasses.xlsx
+++ b/Design files/Left-Side/BOM/Client BOM-LEFT-Bone_Conduction_Glasses.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="144">
   <si>
     <t>#</t>
   </si>
@@ -448,6 +448,9 @@
   </si>
   <si>
     <t>Transducer (GD02)</t>
+  </si>
+  <si>
+    <t>Touch Material</t>
   </si>
 </sst>
 </file>
@@ -988,7 +991,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1093,7 +1096,7 @@
     <row r="4" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B27" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B28" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -1121,7 +1124,7 @@
         <v>18</v>
       </c>
       <c r="K4" s="7">
-        <f t="shared" ref="K4:K28" si="1">J4*5</f>
+        <f t="shared" ref="K4:K26" si="1">J4*5</f>
         <v>90</v>
       </c>
       <c r="L4" s="9"/>
@@ -1953,40 +1956,73 @@
       </c>
       <c r="L27" s="9"/>
     </row>
-    <row r="28" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
-        <f>ROW(B28) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="7"/>
+      <c r="F28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="J28" s="9">
+        <v>1</v>
+      </c>
+      <c r="K28" s="7">
+        <v>5</v>
+      </c>
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="11">
+        <f>ROW(B29) - ROW($B$2)</f>
+        <v>27</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="E29" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="F29" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="G28" s="15" t="s">
+      <c r="G29" s="15" t="s">
         <v>142</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="H29" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="I28" s="16" t="s">
+      <c r="I29" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="J28" s="15">
+      <c r="J29" s="15">
         <v>1</v>
       </c>
-      <c r="K28" s="15">
+      <c r="K29" s="15">
         <v>5</v>
       </c>
-      <c r="L28" s="15"/>
+      <c r="L29" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>